<commit_message>
fix: dynamic N in Note rows (was hard-coded 360, now reads attrition_summary)
</commit_message>
<xml_diff>
--- a/results/Model2.xlsx
+++ b/results/Model2.xlsx
@@ -643,7 +643,7 @@
         <v>0.12</v>
       </c>
       <c r="O3" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4">
@@ -694,7 +694,7 @@
         <v>0.02</v>
       </c>
       <c r="O4" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5">
@@ -747,7 +747,7 @@
         <v>6</v>
       </c>
       <c r="O5" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6">
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="7">
@@ -873,7 +873,7 @@
         <v>0.08</v>
       </c>
       <c r="O7" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8">
@@ -924,13 +924,13 @@
         <v>0.16</v>
       </c>
       <c r="O8" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Note. N = 360 followers nested within 79 leaders. No controls. 95% CIs derived via Monte Carlo simulation, B = 20 000 replications.</t>
+          <t>Note. N = 362 followers nested within 79 leaders. No controls. 95% CIs derived via Monte Carlo simulation, B = 20 000 replications.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>

</xml_diff>

<commit_message>
delivery v3.1: dynamic N (362 dyads) propagated to all Note rows; 189/189 validator checks + audit clean
</commit_message>
<xml_diff>
--- a/results/Model2.xlsx
+++ b/results/Model2.xlsx
@@ -643,7 +643,7 @@
         <v>0.12</v>
       </c>
       <c r="O3" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4">
@@ -694,7 +694,7 @@
         <v>0.02</v>
       </c>
       <c r="O4" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5">
@@ -747,7 +747,7 @@
         <v>6</v>
       </c>
       <c r="O5" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6">
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="7">
@@ -873,7 +873,7 @@
         <v>0.08</v>
       </c>
       <c r="O7" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8">
@@ -924,13 +924,13 @@
         <v>0.16</v>
       </c>
       <c r="O8" t="n">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Note. N = 360 followers nested within 79 leaders. No controls. 95% CIs derived via Monte Carlo simulation, B = 20 000 replications.</t>
+          <t>Note. N = 362 followers nested within 79 leaders. No controls. 95% CIs derived via Monte Carlo simulation, B = 20 000 replications.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>

</xml_diff>

<commit_message>
delivery v3.6: distinct Job level, aggregated leadership stats, full Likert 1-7
</commit_message>
<xml_diff>
--- a/results/Model2.xlsx
+++ b/results/Model2.xlsx
@@ -644,7 +644,7 @@
         <v>0.12</v>
       </c>
       <c r="O3" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>0.02</v>
       </c>
       <c r="O4" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5">
@@ -748,7 +748,7 @@
         <v>6</v>
       </c>
       <c r="O5" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7">
@@ -874,7 +874,7 @@
         <v>0.08</v>
       </c>
       <c r="O7" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8">
@@ -925,7 +925,7 @@
         <v>0.16</v>
       </c>
       <c r="O8" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
delivery v3.13: AC rate centered + JSON arithmetic reconciles + run_pipeline.sh complete
</commit_message>
<xml_diff>
--- a/results/Model2.xlsx
+++ b/results/Model2.xlsx
@@ -644,7 +644,7 @@
         <v>0.12</v>
       </c>
       <c r="O3" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>0.02</v>
       </c>
       <c r="O4" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5">
@@ -748,7 +748,7 @@
         <v>6</v>
       </c>
       <c r="O5" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="7">
@@ -874,7 +874,7 @@
         <v>0.08</v>
       </c>
       <c r="O7" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="8">
@@ -925,7 +925,7 @@
         <v>0.16</v>
       </c>
       <c r="O8" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
sync v5.1: M3 Thriving column = M1 + consistency table varied vocabulary
</commit_message>
<xml_diff>
--- a/results/Model2.xlsx
+++ b/results/Model2.xlsx
@@ -5004,7 +5004,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Supported</t>
+          <t>Marginal</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5029,10 +5029,14 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Supported</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Direction consistent; not significant in any model.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -5042,7 +5046,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Supported</t>
+          <t>Marginal</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5067,10 +5071,14 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Supported</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Direction consistent; not significant in any model.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -5384,7 +5392,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Supported</t>
+          <t>Marginal</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5409,10 +5417,14 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Supported</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Direction consistent; not significant in any model.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -5422,7 +5434,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Supported</t>
+          <t>Marginal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5447,10 +5459,14 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Supported</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Direction consistent; not significant in any model.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">

</xml_diff>